<commit_message>
chinh sua data va database
</commit_message>
<xml_diff>
--- a/Data/Data.xlsx
+++ b/Data/Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thinh Phat\Documents\UIT\MovieManager\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC808623-1A19-4B1D-886D-DBB4CCDE61B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F797F763-E52C-4075-9C57-6D6891ADC57C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{8A1C6B9F-F696-49BA-8ECA-23D238E7B1A7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="10" xr2:uid="{8A1C6B9F-F696-49BA-8ECA-23D238E7B1A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Movie" sheetId="1" r:id="rId1"/>
@@ -19,12 +19,12 @@
     <sheet name="Seat" sheetId="6" r:id="rId4"/>
     <sheet name="Customer" sheetId="7" r:id="rId5"/>
     <sheet name="Shift Schedule" sheetId="8" r:id="rId6"/>
-    <sheet name="Staff" sheetId="9" r:id="rId7"/>
-    <sheet name="Snack" sheetId="10" r:id="rId8"/>
-    <sheet name="ShowTime" sheetId="11" r:id="rId9"/>
-    <sheet name="Ticket" sheetId="12" r:id="rId10"/>
-    <sheet name="Ticket Snack" sheetId="13" r:id="rId11"/>
-    <sheet name="Account" sheetId="14" r:id="rId12"/>
+    <sheet name="Snack" sheetId="10" r:id="rId7"/>
+    <sheet name="ShowTime" sheetId="11" r:id="rId8"/>
+    <sheet name="Ticket" sheetId="12" r:id="rId9"/>
+    <sheet name="Ticket Snack" sheetId="13" r:id="rId10"/>
+    <sheet name="Account" sheetId="14" r:id="rId11"/>
+    <sheet name="Staff" sheetId="9" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="187">
   <si>
     <t>title</t>
   </si>
@@ -91,9 +91,6 @@
     <t>capacity</t>
   </si>
   <si>
-    <t>available seat</t>
-  </si>
-  <si>
     <t>type</t>
   </si>
   <si>
@@ -442,12 +439,6 @@
     <t>Khoai tây chiên</t>
   </si>
   <si>
-    <t>đồ ăn</t>
-  </si>
-  <si>
-    <t>nước uống</t>
-  </si>
-  <si>
     <t>Nguyễn Minh Anh</t>
   </si>
   <si>
@@ -614,6 +605,9 @@
   </si>
   <si>
     <t>Tiếng Indonesia - phụ đề Tiếng Việt, Tiếng Anh</t>
+  </si>
+  <si>
+    <t>brief</t>
   </si>
 </sst>
 </file>
@@ -1076,26 +1070,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB97CE34-ECB9-4A61-9147-3878E4574496}">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.90625" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.54296875" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.453125" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.26953125" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.453125" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="43.90625" style="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8" style="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.54296875" style="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="29.453125" style="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="100.54296875" style="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.08984375" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.1796875" style="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.7265625" style="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.90625" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.6328125" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.7265625" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="49.1796875" style="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.81640625" style="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7" style="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31" style="11" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="137.08984375" style="11" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="8.7265625" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" s="16" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>0</v>
@@ -1125,333 +1119,336 @@
         <v>8</v>
       </c>
       <c r="K1" s="16" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+        <v>100</v>
+      </c>
+      <c r="L1" s="16" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="11">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>49</v>
       </c>
       <c r="E2" s="5">
         <v>45940</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H2" s="2">
         <v>104</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="K2" s="18" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="11">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="G3" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="11">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>61</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>62</v>
       </c>
       <c r="H4" s="2">
         <v>118</v>
       </c>
       <c r="I4" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J4" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="J4" s="8" t="s">
-        <v>64</v>
-      </c>
       <c r="K4" s="18" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="11">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>66</v>
       </c>
       <c r="E5" s="5">
         <v>46000</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H5" s="2">
         <v>136</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K5" s="18" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="11">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>73</v>
-      </c>
       <c r="G6" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H6" s="4">
         <v>118</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K6" s="18" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="11">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>77</v>
-      </c>
       <c r="G7" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H7" s="2">
         <v>95</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K7" s="18" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="11">
         <v>7</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E8" s="20">
         <v>45849</v>
       </c>
       <c r="F8" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="G8" s="18" t="s">
         <v>185</v>
-      </c>
-      <c r="G8" s="18" t="s">
-        <v>188</v>
       </c>
       <c r="H8" s="2">
         <v>98</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="17" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="K8" s="18" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="E9" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>83</v>
-      </c>
       <c r="G9" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H9" s="2">
         <v>119</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K9" s="18" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="11">
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K10" s="18" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>94</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="K11" s="18" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -1472,43 +1469,40 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E19FF20-36A3-40D1-8B97-3AF311333246}">
-  <dimension ref="A1:K1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C23B777-4B0C-44AB-9E85-F8473D6A4A84}">
+  <dimension ref="A1:L1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="9" max="9" width="2.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.90625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.54296875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>95</v>
       </c>
       <c r="B1" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="C1" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
+        <v>95</v>
+      </c>
+      <c r="J1" t="s">
+        <v>175</v>
+      </c>
+      <c r="K1" t="s">
         <v>38</v>
       </c>
-      <c r="J1" t="s">
-        <v>39</v>
-      </c>
-      <c r="K1" t="s">
-        <v>40</v>
+      <c r="L1" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1517,42 +1511,6 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C23B777-4B0C-44AB-9E85-F8473D6A4A84}">
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" t="s">
-        <v>42</v>
-      </c>
-      <c r="I1" t="s">
-        <v>96</v>
-      </c>
-      <c r="J1" t="s">
-        <v>178</v>
-      </c>
-      <c r="K1" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AF3BE82-C9F8-48B6-B4D9-D671358516C3}">
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1566,19 +1524,19 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B1" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="D1" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="11" t="s">
-        <v>45</v>
-      </c>
       <c r="E1" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -1586,10 +1544,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D2" s="11">
         <v>1</v>
@@ -1607,10 +1565,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D3" s="11">
         <v>0</v>
@@ -1628,10 +1586,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D4" s="11">
         <v>1</v>
@@ -1649,10 +1607,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D5" s="11">
         <v>1</v>
@@ -1670,10 +1628,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D6" s="11">
         <v>0</v>
@@ -1691,10 +1649,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D7" s="11">
         <v>0</v>
@@ -1712,10 +1670,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D8" s="11">
         <v>0</v>
@@ -1742,595 +1700,152 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91837C5C-D31D-4D0B-8F0E-95A94197B1D7}">
-  <dimension ref="A1:C6"/>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1372C545-3A1C-4A65-85EA-5A0B149575F3}">
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="105.81640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="9">
-        <v>1</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="9">
-        <v>2</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="9">
-        <v>3</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="9">
-        <v>4</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="9">
-        <v>5</v>
-      </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC35A546-C17F-4306-B513-4D44EE24DE6C}">
-  <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E51C45A-0E1C-4B96-B5C6-16961647AD7C}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08637C6E-015B-4C98-AA0C-5F1E03F281FF}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="4" max="4" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B1" t="s">
         <v>9</v>
       </c>
       <c r="C1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68B02B28-5C9A-4FD1-9513-1298E635070B}">
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="12.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7265625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="15" t="s">
-        <v>173</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>174</v>
-      </c>
-      <c r="E2" s="14" t="str">
-        <f>"INSERT INTO dbo.Shift_Schedule VALUES('"&amp;B2&amp;"', '"&amp;C2&amp;"');"</f>
-        <v>INSERT INTO dbo.Shift_Schedule VALUES('7:30:00', '12:30:00');</v>
+      <c r="B2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="15" t="s">
-        <v>174</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>175</v>
-      </c>
-      <c r="E3" s="14" t="str">
-        <f t="shared" ref="E3:E5" si="0">"INSERT INTO dbo.Shift_Schedule VALUES('"&amp;B3&amp;"', '"&amp;C3&amp;"');"</f>
-        <v>INSERT INTO dbo.Shift_Schedule VALUES('12:30:00', '17:30:00');</v>
+      <c r="B3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="15" t="s">
-        <v>175</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="E4" s="14" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO dbo.Shift_Schedule VALUES('17:30:00', '22:30:00');</v>
+      <c r="B4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C4" t="s">
+        <v>135</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>177</v>
-      </c>
-      <c r="E5" s="14" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO dbo.Shift_Schedule VALUES('22:30:00', '2:30:00');</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B7" s="15"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1372C545-3A1C-4A65-85EA-5A0B149575F3}">
-  <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.54296875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>133</v>
-      </c>
-      <c r="C2" t="s">
-        <v>134</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="G2" t="str">
-        <f>"INSERT INTO dbo.Staff VALUES('"&amp;B2&amp;"', '"&amp;C2&amp;"', '"&amp;D2&amp;"', '"&amp;E2&amp;"');"</f>
-        <v>INSERT INTO dbo.Staff VALUES('Nguyễn Minh Anh', 'Giám đốc marketing', 'mlanhmlanh214@gmail.com', '1');</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="B5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C5" t="s">
         <v>135</v>
       </c>
-      <c r="C3" t="s">
-        <v>136</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="G3" t="str">
-        <f t="shared" ref="G3:G8" si="0">"INSERT INTO dbo.Staff VALUES('"&amp;B3&amp;"', '"&amp;C3&amp;"', '"&amp;D3&amp;"', '"&amp;E3&amp;"');"</f>
-        <v>INSERT INTO dbo.Staff VALUES('Trần Minh Đức', 'Nhân viên', 'minhduct50@gmail.com', '1');</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>137</v>
-      </c>
-      <c r="C4" t="s">
-        <v>138</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="G4" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO dbo.Staff VALUES('Phạm Đan Trường', 'Quản lý', 'truongpd.a2.2124@gmail.com', '1');</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>139</v>
-      </c>
-      <c r="C5" t="s">
-        <v>138</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E5">
         <v>3</v>
       </c>
-      <c r="G5" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO dbo.Staff VALUES('Hồ Thịnh Phát', 'Quản lý', 'phatht.a2.2124@gmail.com', '3');</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C6" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E6">
         <v>2</v>
       </c>
-      <c r="G6" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO dbo.Staff VALUES('Võ Việt Thy', 'Nhân viên', 'thyvv.a2.2124@gmail.com', '2');</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C7" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E7">
         <v>3</v>
       </c>
-      <c r="G7" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO dbo.Staff VALUES('Lê Phương Thúy', 'Nhân viên', 'thuylp.a2.2124@gmail.com', '3');</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C8" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E8">
         <v>4</v>
-      </c>
-      <c r="G8" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO dbo.Staff VALUES('Nguyễn Thanh Hiếu Thảo', 'Nhân viên', 'thaontt.a2.2124@gmail.com', '4');</v>
       </c>
     </row>
   </sheetData>
@@ -2347,33 +1862,554 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91837C5C-D31D-4D0B-8F0E-95A94197B1D7}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="2.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="97.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC35A546-C17F-4306-B513-4D44EE24DE6C}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="2.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E51C45A-0E1C-4B96-B5C6-16961647AD7C}">
+  <dimension ref="A1:E51"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08637C6E-015B-4C98-AA0C-5F1E03F281FF}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="2.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68B02B28-5C9A-4FD1-9513-1298E635070B}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="2.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="E2" s="14"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="E3" s="14"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="E4" s="14"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="E5" s="14"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B7" s="15"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A5FDDEC-2C27-4D76-B8E2-D224C508B564}">
   <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.90625" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.90625" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="8.7265625" style="12"/>
-    <col min="5" max="5" width="9.36328125" style="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.453125" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.08984375" style="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.7265625" style="12" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="8.7265625" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -2381,7 +2417,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C2" s="12">
         <v>55000</v>
@@ -2389,8 +2425,8 @@
       <c r="D2" s="12">
         <v>100</v>
       </c>
-      <c r="E2" s="12" t="s">
-        <v>131</v>
+      <c r="E2" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -2398,7 +2434,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C3" s="12">
         <v>59000</v>
@@ -2406,8 +2442,8 @@
       <c r="D3" s="12">
         <v>100</v>
       </c>
-      <c r="E3" s="12" t="s">
-        <v>131</v>
+      <c r="E3" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -2415,7 +2451,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C4" s="12">
         <v>59000</v>
@@ -2423,8 +2459,8 @@
       <c r="D4" s="12">
         <v>100</v>
       </c>
-      <c r="E4" s="12" t="s">
-        <v>131</v>
+      <c r="E4" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -2432,7 +2468,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C5" s="12">
         <v>39000</v>
@@ -2440,8 +2476,8 @@
       <c r="D5" s="12">
         <v>100</v>
       </c>
-      <c r="E5" s="12" t="s">
-        <v>131</v>
+      <c r="E5" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -2449,7 +2485,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C6" s="12">
         <v>19000</v>
@@ -2457,8 +2493,8 @@
       <c r="D6" s="12">
         <v>100</v>
       </c>
-      <c r="E6" s="12" t="s">
-        <v>131</v>
+      <c r="E6" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -2466,7 +2502,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12">
         <v>49000</v>
@@ -2474,8 +2510,8 @@
       <c r="D7" s="12">
         <v>100</v>
       </c>
-      <c r="E7" s="12" t="s">
-        <v>131</v>
+      <c r="E7" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -2483,7 +2519,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C8" s="12">
         <v>39000</v>
@@ -2491,8 +2527,8 @@
       <c r="D8" s="12">
         <v>100</v>
       </c>
-      <c r="E8" s="12" t="s">
-        <v>132</v>
+      <c r="E8" s="12">
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -2500,7 +2536,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C9" s="12">
         <v>39000</v>
@@ -2508,8 +2544,8 @@
       <c r="D9" s="12">
         <v>100</v>
       </c>
-      <c r="E9" s="12" t="s">
-        <v>132</v>
+      <c r="E9" s="12">
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -2517,7 +2553,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C10" s="12">
         <v>39000</v>
@@ -2525,8 +2561,8 @@
       <c r="D10" s="12">
         <v>100</v>
       </c>
-      <c r="E10" s="12" t="s">
-        <v>132</v>
+      <c r="E10" s="12">
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -2534,7 +2570,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C11" s="12">
         <v>39000</v>
@@ -2542,8 +2578,8 @@
       <c r="D11" s="12">
         <v>100</v>
       </c>
-      <c r="E11" s="12" t="s">
-        <v>132</v>
+      <c r="E11" s="12">
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -2551,7 +2587,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C12" s="12">
         <v>49000</v>
@@ -2559,8 +2595,8 @@
       <c r="D12" s="12">
         <v>100</v>
       </c>
-      <c r="E12" s="12" t="s">
-        <v>132</v>
+      <c r="E12" s="12">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -2568,7 +2604,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C13" s="12">
         <v>49000</v>
@@ -2576,8 +2612,8 @@
       <c r="D13" s="12">
         <v>100</v>
       </c>
-      <c r="E13" s="12" t="s">
-        <v>132</v>
+      <c r="E13" s="12">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -2585,7 +2621,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C14" s="12">
         <v>39000</v>
@@ -2593,8 +2629,8 @@
       <c r="D14" s="12">
         <v>100</v>
       </c>
-      <c r="E14" s="12" t="s">
-        <v>132</v>
+      <c r="E14" s="12">
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -2602,7 +2638,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C15" s="12">
         <v>49000</v>
@@ -2610,8 +2646,8 @@
       <c r="D15" s="12">
         <v>100</v>
       </c>
-      <c r="E15" s="12" t="s">
-        <v>132</v>
+      <c r="E15" s="12">
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -2619,7 +2655,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C16" s="12">
         <v>25000</v>
@@ -2627,8 +2663,8 @@
       <c r="D16" s="12">
         <v>100</v>
       </c>
-      <c r="E16" s="12" t="s">
-        <v>131</v>
+      <c r="E16" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -2636,7 +2672,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C17" s="12">
         <v>39000</v>
@@ -2644,8 +2680,8 @@
       <c r="D17" s="12">
         <v>100</v>
       </c>
-      <c r="E17" s="12" t="s">
-        <v>131</v>
+      <c r="E17" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -2653,7 +2689,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C18" s="12">
         <v>55000</v>
@@ -2661,8 +2697,8 @@
       <c r="D18" s="12">
         <v>100</v>
       </c>
-      <c r="E18" s="12" t="s">
-        <v>131</v>
+      <c r="E18" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -2670,7 +2706,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C19" s="12">
         <v>39000</v>
@@ -2678,8 +2714,8 @@
       <c r="D19" s="12">
         <v>100</v>
       </c>
-      <c r="E19" s="12" t="s">
-        <v>131</v>
+      <c r="E19" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -2687,7 +2723,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C20" s="12">
         <v>39000</v>
@@ -2695,8 +2731,8 @@
       <c r="D20" s="12">
         <v>100</v>
       </c>
-      <c r="E20" s="12" t="s">
-        <v>131</v>
+      <c r="E20" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -2704,7 +2740,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C21" s="12">
         <v>35000</v>
@@ -2712,8 +2748,8 @@
       <c r="D21" s="12">
         <v>100</v>
       </c>
-      <c r="E21" s="12" t="s">
-        <v>131</v>
+      <c r="E21" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
@@ -2721,7 +2757,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C22" s="12">
         <v>49000</v>
@@ -2729,8 +2765,8 @@
       <c r="D22" s="12">
         <v>100</v>
       </c>
-      <c r="E22" s="12" t="s">
-        <v>131</v>
+      <c r="E22" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
@@ -2738,7 +2774,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C23" s="12">
         <v>5000</v>
@@ -2746,8 +2782,8 @@
       <c r="D23" s="12">
         <v>100</v>
       </c>
-      <c r="E23" s="12" t="s">
-        <v>131</v>
+      <c r="E23" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
@@ -2755,7 +2791,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C24" s="12">
         <v>59000</v>
@@ -2763,8 +2799,8 @@
       <c r="D24" s="12">
         <v>100</v>
       </c>
-      <c r="E24" s="12" t="s">
-        <v>131</v>
+      <c r="E24" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
@@ -2772,7 +2808,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C25" s="12">
         <v>65000</v>
@@ -2780,8 +2816,8 @@
       <c r="D25" s="12">
         <v>100</v>
       </c>
-      <c r="E25" s="12" t="s">
-        <v>131</v>
+      <c r="E25" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
@@ -2789,7 +2825,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C26" s="12">
         <v>65000</v>
@@ -2797,8 +2833,46 @@
       <c r="D26" s="12">
         <v>100</v>
       </c>
-      <c r="E26" s="12" t="s">
-        <v>131</v>
+      <c r="E26" s="12">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E26EBFAF-9DA8-4EDC-9279-5B2C28B4541B}">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="2.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -2807,28 +2881,43 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E26EBFAF-9DA8-4EDC-9279-5B2C28B4541B}">
-  <dimension ref="A1:F1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E19FF20-36A3-40D1-8B97-3AF311333246}">
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>96</v>
+        <v>26</v>
       </c>
       <c r="B1" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>31</v>
+        <v>95</v>
+      </c>
+      <c r="G1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" t="s">
+        <v>36</v>
+      </c>
+      <c r="I1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K1" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>